<commit_message>
refactor: Consolidate 24-sheet master model, remove duplicate Observaciones, update Geofencing formula to [ActivoID].[Ubicacion] and update Audit-First prompt
</commit_message>
<xml_diff>
--- a/BD/Modelo de Datos (2).xlsx
+++ b/BD/Modelo de Datos (2).xlsx
@@ -4743,7 +4743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="7.29" customWidth="1" style="40" min="1" max="1"/>
@@ -4773,132 +4773,128 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>MantenimientoID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OTID</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ActivoID</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>TécnicoID</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Hora Inicio</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Hora Fin</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Estado Final</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Coordenadas_Cierre</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Precision_GPS</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Requiere_Segunda_Visita</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Motivo_Pendiente</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Estado_Intervencion</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Localizacion</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Imagen_Inicio</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Imagen_Final</t>
         </is>
       </c>
-      <c r="S1" s="7" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
-      </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Firma_Tecnico</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Firma_Supervisor</t>
         </is>
       </c>
-      <c r="V1" s="7" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Aprobado_Supervisor</t>
         </is>
       </c>
-      <c r="W1" s="7" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Usuario_Registro</t>
         </is>
       </c>
-      <c r="X1" s="7" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Fecha_Hora_Registro</t>
         </is>
       </c>
-      <c r="Y1" s="7" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="19" ht="15.75" customHeight="1" s="40"/>
     <row r="20" ht="15.75" customHeight="1" s="40"/>
     <row r="21" ht="15.75" customHeight="1" s="40"/>

</xml_diff>